<commit_message>
GerberX2 datei der Hauptplatine hinzugefügt + BOM
</commit_message>
<xml_diff>
--- a/BOM/BOM.xlsx
+++ b/BOM/BOM.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="DieseArbeitsmappe"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abdul\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abdul\Documents\GITHUB\3D-Display\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FA057144-074F-4087-B45F-2D8AD6A94C34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A8CAC5C-9F7C-43B8-803B-8BB8B79F8E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="384">
   <si>
     <t>Best.</t>
   </si>
@@ -581,6 +581,9 @@
     <t>CAP CER 1UF 16V X5R 0603</t>
   </si>
   <si>
+    <t>Connector</t>
+  </si>
+  <si>
     <t>RES 13.7K OHM 1/8W .1% SMD 0805</t>
   </si>
   <si>
@@ -846,6 +849,357 @@
   </si>
   <si>
     <t>VDPG</t>
+  </si>
+  <si>
+    <t>VPDM</t>
+  </si>
+  <si>
+    <t>VDPH</t>
+  </si>
+  <si>
+    <t>Hallsensor</t>
+  </si>
+  <si>
+    <t>595-MAG5170A2EDGKRQ1</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4vYiBPX</t>
+  </si>
+  <si>
+    <t>77-VJ0805Y104JXXPBC</t>
+  </si>
+  <si>
+    <t>https://mou.sr/3SVcb5s</t>
+  </si>
+  <si>
+    <t>80-C0805C475K3RAUTO</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4vuBBo7</t>
+  </si>
+  <si>
+    <t>CAP CER 4,7nF 0805</t>
+  </si>
+  <si>
+    <t>603-CC805KKX7R5BB105</t>
+  </si>
+  <si>
+    <t>CAP CER 1uF 0805</t>
+  </si>
+  <si>
+    <t>https://mou.sr/3RzsAfr</t>
+  </si>
+  <si>
+    <t>603-AC805KRX7R0BB103</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4pil6tK</t>
+  </si>
+  <si>
+    <t>CAP CER 10nF 0805</t>
+  </si>
+  <si>
+    <t>581-0805ZC106KAT2A</t>
+  </si>
+  <si>
+    <t>https://mou.sr/44ZwIIE</t>
+  </si>
+  <si>
+    <t>CAP CER 10uF 0805</t>
+  </si>
+  <si>
+    <t>CAP CER 470nF 0805</t>
+  </si>
+  <si>
+    <t>80-C0805C474J3RAUTO</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4vX50bj</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4fgtJR1</t>
+  </si>
+  <si>
+    <t>81-GRM21BR61E106MA3L</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4vAmZUk</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4bgyqZO</t>
+  </si>
+  <si>
+    <t>810-CGA4J2X7R1C105KD</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4f9QXrI</t>
+  </si>
+  <si>
+    <t>CAP CER 1uF</t>
+  </si>
+  <si>
+    <t>81-KRM55QR71E336KH1L</t>
+  </si>
+  <si>
+    <t>Cap Ceramic 33uF 25V X7R</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4ymUcoS</t>
+  </si>
+  <si>
+    <t>80-C1206C473K5H</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4vuCLQv</t>
+  </si>
+  <si>
+    <t>CAP Cer 47nF</t>
+  </si>
+  <si>
+    <t>771-74AHCT245APWJ</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4vsnobd</t>
+  </si>
+  <si>
+    <t>Bustransceiver</t>
+  </si>
+  <si>
+    <t>700-MAX17320G20+</t>
+  </si>
+  <si>
+    <t>BatteryManagement</t>
+  </si>
+  <si>
+    <t>https://mou.sr/3SVeaGW</t>
+  </si>
+  <si>
+    <t>512-FDC608PZ</t>
+  </si>
+  <si>
+    <t>Mosfet P-Channel</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4feU6Xy</t>
+  </si>
+  <si>
+    <t>Sockel</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4wGJvvF</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4bBXdHM</t>
+  </si>
+  <si>
+    <t>SD-Kartenleser</t>
+  </si>
+  <si>
+    <t>179-MSD-5-A</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4bAGjJC</t>
+  </si>
+  <si>
+    <t>710-629722000214</t>
+  </si>
+  <si>
+    <t>https://mou.sr/3R1WMzH</t>
+  </si>
+  <si>
+    <t>USB-C Socket</t>
+  </si>
+  <si>
+    <t>710-74479332257210</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4fgvHkt</t>
+  </si>
+  <si>
+    <t>Spule 1uH</t>
+  </si>
+  <si>
+    <t>720-LGR971-KN-1</t>
+  </si>
+  <si>
+    <t>https://mou.sr/44on16s</t>
+  </si>
+  <si>
+    <t>LED</t>
+  </si>
+  <si>
+    <t>726-IRF7313TRPBFXTMA</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4vYljVD</t>
+  </si>
+  <si>
+    <t>Mosfet N-Channel</t>
+  </si>
+  <si>
+    <t>71-PCAN0805E1001BST5</t>
+  </si>
+  <si>
+    <t>https://mou.sr/44oh75q</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4ylH4QQ</t>
+  </si>
+  <si>
+    <t>279-CRGP1206F47R</t>
+  </si>
+  <si>
+    <t>Res 47R Dickfilm</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4vsouUn</t>
+  </si>
+  <si>
+    <t>https://mou.sr/3TfI8FD</t>
+  </si>
+  <si>
+    <t>Res 22k1</t>
+  </si>
+  <si>
+    <t>660-RN73R2ATD1000B25</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4wApiau</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Res 100Ω 0805 </t>
+  </si>
+  <si>
+    <t>708-RMCF0805JT560R</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4fvOZU1</t>
+  </si>
+  <si>
+    <t>Res 560R 0805</t>
+  </si>
+  <si>
+    <t>660-RK73H2ATTDD1503F</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4pinNLS</t>
+  </si>
+  <si>
+    <t>Res 150k 0805</t>
+  </si>
+  <si>
+    <t>279-RP73PF2A5K23BTDF</t>
+  </si>
+  <si>
+    <t>https://mou.sr/44Ybivy</t>
+  </si>
+  <si>
+    <t>Res 5k23 0805</t>
+  </si>
+  <si>
+    <t>603-RC0805FR-075K76L</t>
+  </si>
+  <si>
+    <t>https://mou.sr/3Teegtb</t>
+  </si>
+  <si>
+    <t>Res 5k76 0805</t>
+  </si>
+  <si>
+    <t>954-103AT-2</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4vZiUty</t>
+  </si>
+  <si>
+    <t>Thermresistoren NTC</t>
+  </si>
+  <si>
+    <t>594-MCU08050D3012BP1</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4ygmhOh</t>
+  </si>
+  <si>
+    <t>Res 30k1 0805</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4pdbdxg</t>
+  </si>
+  <si>
+    <t>Res 13k7 0805</t>
+  </si>
+  <si>
+    <t>603-RC0805FR-07383RL</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4h84vGX</t>
+  </si>
+  <si>
+    <t>Res 383R 0805 Dickmann</t>
+  </si>
+  <si>
+    <t>603-AC0805JR-075K1L</t>
+  </si>
+  <si>
+    <t>https://mou.sr/3QStgfM</t>
+  </si>
+  <si>
+    <t>Res 5k1 0805</t>
+  </si>
+  <si>
+    <t>603-RC0805JR-134K7L</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4pdFpbI</t>
+  </si>
+  <si>
+    <t>Res 4k7 0805</t>
+  </si>
+  <si>
+    <t>Switch</t>
+  </si>
+  <si>
+    <t>229-CFS-0102TA</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4wH3bzu</t>
+  </si>
+  <si>
+    <t>511-STM32G431CBT6</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4w5ykgc</t>
+  </si>
+  <si>
+    <t>STM32G431CBT6</t>
+  </si>
+  <si>
+    <t>595-BQ25886RGER</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4aMSoeD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boost Battery </t>
+  </si>
+  <si>
+    <t>conrad</t>
+  </si>
+  <si>
+    <t>740197 - UP</t>
+  </si>
+  <si>
+    <t>https://www.conrad.at/de/p/jst-einbau-stiftleiste-standard-ph-polzahl-gesamt-2-rastermass-2-mm-s2b-ph-k-s-lf-sn-1-st-740197.html?srsltid=AfmBOooo9BOmWD_uhxWb4a2mY14-Qu3-5fNR4kmU1FAuQtNaVtE351Be</t>
+  </si>
+  <si>
+    <t>71-WSHP28185L000FEA</t>
+  </si>
+  <si>
+    <t>https://mou.sr/4wXNu7h</t>
+  </si>
+  <si>
+    <t>Strommesswiderstand</t>
   </si>
 </sst>
 </file>
@@ -858,7 +1212,7 @@
     <numFmt numFmtId="166" formatCode="0.0\ &quot;kg&quot;"/>
     <numFmt numFmtId="167" formatCode="_-* #,##0.0000\ &quot;€&quot;_-;\-* #,##0.0000\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -896,6 +1250,12 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="6"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <u/>
       <sz val="11"/>
       <color theme="1"/>
@@ -912,7 +1272,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -949,13 +1309,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -990,9 +1359,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1003,13 +1369,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Link" xfId="2" builtinId="8"/>
@@ -1293,7 +1661,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Tabelle1"/>
-  <dimension ref="A1:O64"/>
+  <dimension ref="A1:O92"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.3984375" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="7.73046875" bestFit="1" customWidth="1"/>
@@ -1301,7 +1669,7 @@
     <col min="4" max="4" width="13" customWidth="1"/>
     <col min="5" max="5" width="19.73046875" customWidth="1"/>
     <col min="6" max="6" width="28" customWidth="1"/>
-    <col min="7" max="7" width="10.73046875" style="28" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.73046875" style="27" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.73046875" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14.59765625" bestFit="1" customWidth="1"/>
@@ -1314,18 +1682,18 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A1" s="10" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="G2" s="29"/>
+      <c r="G2" s="28"/>
       <c r="H2" s="10"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.45">
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="31" t="s">
+      <c r="C3" s="30" t="s">
         <v>1</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -1337,7 +1705,7 @@
       <c r="F3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="34" t="s">
+      <c r="G3" s="33" t="s">
         <v>5</v>
       </c>
       <c r="H3" s="1" t="s">
@@ -1367,21 +1735,21 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
-        <v>263</v>
-      </c>
-      <c r="C4" s="32" t="s">
-        <v>181</v>
+        <v>267</v>
+      </c>
+      <c r="C4" s="31" t="s">
+        <v>182</v>
       </c>
       <c r="D4" t="s">
-        <v>185</v>
-      </c>
-      <c r="E4" s="32" t="s">
-        <v>209</v>
+        <v>186</v>
+      </c>
+      <c r="E4" s="31" t="s">
+        <v>210</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>210</v>
-      </c>
-      <c r="G4" s="33">
+        <v>211</v>
+      </c>
+      <c r="G4" s="32">
         <v>2</v>
       </c>
       <c r="I4" s="14">
@@ -1395,7 +1763,7 @@
         <f>I4*G4</f>
         <v>0.312</v>
       </c>
-      <c r="L4" s="25">
+      <c r="L4" s="24">
         <f>J4*G4</f>
         <v>0.26</v>
       </c>
@@ -1404,22 +1772,22 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
-        <v>263</v>
-      </c>
-      <c r="C5" s="32" t="s">
-        <v>180</v>
+        <v>264</v>
+      </c>
+      <c r="C5" s="31" t="s">
+        <v>181</v>
       </c>
       <c r="D5" t="s">
-        <v>185</v>
-      </c>
-      <c r="E5" s="32" t="s">
-        <v>211</v>
+        <v>186</v>
+      </c>
+      <c r="E5" s="31" t="s">
+        <v>212</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>212</v>
-      </c>
-      <c r="G5" s="33">
-        <v>4</v>
+        <v>213</v>
+      </c>
+      <c r="G5" s="32">
+        <v>8</v>
       </c>
       <c r="I5" s="14">
         <f t="shared" ref="I5:I28" si="0">J5*1.2</f>
@@ -1430,32 +1798,32 @@
       </c>
       <c r="K5" s="14">
         <f t="shared" ref="K5:K28" si="1">I5*G5</f>
-        <v>3.36</v>
-      </c>
-      <c r="L5" s="25">
+        <v>6.72</v>
+      </c>
+      <c r="L5" s="24">
         <f t="shared" ref="L5:L28" si="2">J5*G5</f>
-        <v>2.8</v>
+        <v>5.6</v>
       </c>
       <c r="M5" s="16"/>
       <c r="N5" s="15"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
-        <v>263</v>
-      </c>
-      <c r="C6" s="33" t="s">
+        <v>264</v>
+      </c>
+      <c r="C6" s="32" t="s">
+        <v>226</v>
+      </c>
+      <c r="D6" t="s">
+        <v>186</v>
+      </c>
+      <c r="E6" s="31" t="s">
         <v>225</v>
       </c>
-      <c r="D6" t="s">
-        <v>185</v>
-      </c>
-      <c r="E6" s="32" t="s">
+      <c r="F6" s="19" t="s">
         <v>224</v>
       </c>
-      <c r="F6" s="19" t="s">
-        <v>223</v>
-      </c>
-      <c r="G6" s="33">
+      <c r="G6" s="32">
         <v>1</v>
       </c>
       <c r="I6" s="14">
@@ -1469,7 +1837,7 @@
         <f t="shared" si="1"/>
         <v>0.20400000000000001</v>
       </c>
-      <c r="L6" s="25">
+      <c r="L6" s="24">
         <f t="shared" si="2"/>
         <v>0.17</v>
       </c>
@@ -1478,21 +1846,21 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
-        <v>263</v>
-      </c>
-      <c r="C7" s="32" t="s">
-        <v>179</v>
+        <v>264</v>
+      </c>
+      <c r="C7" s="31" t="s">
+        <v>180</v>
       </c>
       <c r="D7" t="s">
-        <v>185</v>
-      </c>
-      <c r="E7" s="32" t="s">
-        <v>213</v>
+        <v>186</v>
+      </c>
+      <c r="E7" s="31" t="s">
+        <v>214</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>214</v>
-      </c>
-      <c r="G7" s="33">
+        <v>215</v>
+      </c>
+      <c r="G7" s="32">
         <v>3</v>
       </c>
       <c r="I7" s="14">
@@ -1506,7 +1874,7 @@
         <f t="shared" si="1"/>
         <v>0.32400000000000001</v>
       </c>
-      <c r="L7" s="25">
+      <c r="L7" s="24">
         <f t="shared" si="2"/>
         <v>0.27</v>
       </c>
@@ -1515,21 +1883,21 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
-        <v>263</v>
-      </c>
-      <c r="C8" s="32" t="s">
+        <v>264</v>
+      </c>
+      <c r="C8" s="31" t="s">
         <v>175</v>
       </c>
       <c r="D8" t="s">
-        <v>185</v>
-      </c>
-      <c r="E8" s="32" t="s">
-        <v>215</v>
+        <v>186</v>
+      </c>
+      <c r="E8" s="31" t="s">
+        <v>216</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>216</v>
-      </c>
-      <c r="G8" s="33">
+        <v>217</v>
+      </c>
+      <c r="G8" s="32">
         <v>2</v>
       </c>
       <c r="I8" s="14">
@@ -1543,7 +1911,7 @@
         <f t="shared" si="1"/>
         <v>0.38400000000000001</v>
       </c>
-      <c r="L8" s="25">
+      <c r="L8" s="24">
         <f t="shared" si="2"/>
         <v>0.32</v>
       </c>
@@ -1552,21 +1920,21 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>263</v>
-      </c>
-      <c r="C9" s="32" t="s">
+        <v>264</v>
+      </c>
+      <c r="C9" s="31" t="s">
         <v>176</v>
       </c>
       <c r="D9" t="s">
-        <v>185</v>
-      </c>
-      <c r="E9" s="32" t="s">
-        <v>217</v>
+        <v>186</v>
+      </c>
+      <c r="E9" s="31" t="s">
+        <v>218</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>218</v>
-      </c>
-      <c r="G9" s="33">
+        <v>219</v>
+      </c>
+      <c r="G9" s="32">
         <v>1</v>
       </c>
       <c r="I9" s="14">
@@ -1580,7 +1948,7 @@
         <f t="shared" si="1"/>
         <v>0.12</v>
       </c>
-      <c r="L9" s="25">
+      <c r="L9" s="24">
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
@@ -1589,21 +1957,21 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
-        <v>263</v>
-      </c>
-      <c r="C10" s="32" t="s">
-        <v>228</v>
+        <v>264</v>
+      </c>
+      <c r="C10" s="31" t="s">
+        <v>229</v>
       </c>
       <c r="D10" t="s">
-        <v>185</v>
-      </c>
-      <c r="E10" s="32" t="s">
+        <v>186</v>
+      </c>
+      <c r="E10" s="31" t="s">
+        <v>231</v>
+      </c>
+      <c r="F10" s="19" t="s">
         <v>230</v>
       </c>
-      <c r="F10" s="19" t="s">
-        <v>229</v>
-      </c>
-      <c r="G10" s="33">
+      <c r="G10" s="32">
         <v>2</v>
       </c>
       <c r="I10" s="14">
@@ -1617,7 +1985,7 @@
         <f t="shared" si="1"/>
         <v>2.2559999999999998</v>
       </c>
-      <c r="L10" s="25">
+      <c r="L10" s="24">
         <f t="shared" si="2"/>
         <v>1.88</v>
       </c>
@@ -1626,21 +1994,21 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
-        <v>263</v>
-      </c>
-      <c r="C11" s="32" t="s">
-        <v>178</v>
+        <v>264</v>
+      </c>
+      <c r="C11" s="31" t="s">
+        <v>179</v>
       </c>
       <c r="D11" t="s">
-        <v>185</v>
-      </c>
-      <c r="E11" s="32" t="s">
-        <v>226</v>
+        <v>186</v>
+      </c>
+      <c r="E11" s="31" t="s">
+        <v>227</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>227</v>
-      </c>
-      <c r="G11" s="33">
+        <v>228</v>
+      </c>
+      <c r="G11" s="32">
         <v>1</v>
       </c>
       <c r="I11" s="14">
@@ -1654,7 +2022,7 @@
         <f t="shared" si="1"/>
         <v>0.13200000000000001</v>
       </c>
-      <c r="L11" s="25">
+      <c r="L11" s="24">
         <f t="shared" si="2"/>
         <v>0.11</v>
       </c>
@@ -1663,22 +2031,22 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
-        <v>263</v>
-      </c>
-      <c r="C12" s="32" t="s">
-        <v>186</v>
+        <v>264</v>
+      </c>
+      <c r="C12" s="31" t="s">
+        <v>187</v>
       </c>
       <c r="D12" t="s">
+        <v>186</v>
+      </c>
+      <c r="E12" s="31" t="s">
         <v>185</v>
       </c>
-      <c r="E12" s="32" t="s">
-        <v>184</v>
-      </c>
       <c r="F12" s="19" t="s">
-        <v>187</v>
-      </c>
-      <c r="G12" s="33">
-        <v>2</v>
+        <v>188</v>
+      </c>
+      <c r="G12" s="32">
+        <v>4</v>
       </c>
       <c r="I12" s="14">
         <f t="shared" si="0"/>
@@ -1689,32 +2057,32 @@
       </c>
       <c r="K12" s="14">
         <f t="shared" si="1"/>
-        <v>3.7919999999999998</v>
-      </c>
-      <c r="L12" s="25">
+        <v>7.5839999999999996</v>
+      </c>
+      <c r="L12" s="24">
         <f t="shared" si="2"/>
-        <v>3.16</v>
+        <v>6.32</v>
       </c>
       <c r="M12" s="16"/>
       <c r="N12" s="15"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
-        <v>263</v>
-      </c>
-      <c r="C13" s="32" t="s">
-        <v>219</v>
+        <v>264</v>
+      </c>
+      <c r="C13" s="31" t="s">
+        <v>220</v>
       </c>
       <c r="D13" t="s">
-        <v>185</v>
-      </c>
-      <c r="E13" s="32" t="s">
-        <v>220</v>
+        <v>186</v>
+      </c>
+      <c r="E13" s="31" t="s">
+        <v>221</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>221</v>
-      </c>
-      <c r="G13" s="33">
+        <v>222</v>
+      </c>
+      <c r="G13" s="32">
         <v>1</v>
       </c>
       <c r="I13" s="14">
@@ -1728,7 +2096,7 @@
         <f t="shared" si="1"/>
         <v>0.72</v>
       </c>
-      <c r="L13" s="25">
+      <c r="L13" s="24">
         <f t="shared" si="2"/>
         <v>0.6</v>
       </c>
@@ -1737,21 +2105,21 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
-        <v>263</v>
-      </c>
-      <c r="C14" s="32" t="s">
-        <v>222</v>
+        <v>264</v>
+      </c>
+      <c r="C14" s="31" t="s">
+        <v>223</v>
       </c>
       <c r="D14" t="s">
-        <v>185</v>
-      </c>
-      <c r="E14" s="32" t="s">
-        <v>189</v>
+        <v>186</v>
+      </c>
+      <c r="E14" s="31" t="s">
+        <v>190</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>190</v>
-      </c>
-      <c r="G14" s="33">
+        <v>191</v>
+      </c>
+      <c r="G14" s="32">
         <v>2</v>
       </c>
       <c r="I14" s="14">
@@ -1765,7 +2133,7 @@
         <f t="shared" si="1"/>
         <v>3.7679999999999998</v>
       </c>
-      <c r="L14" s="25">
+      <c r="L14" s="24">
         <f t="shared" si="2"/>
         <v>3.14</v>
       </c>
@@ -1774,21 +2142,21 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.45">
       <c r="B15" t="s">
-        <v>263</v>
-      </c>
-      <c r="C15" s="32" t="s">
-        <v>188</v>
+        <v>264</v>
+      </c>
+      <c r="C15" s="31" t="s">
+        <v>189</v>
       </c>
       <c r="D15" t="s">
-        <v>185</v>
-      </c>
-      <c r="E15" s="32" t="s">
-        <v>191</v>
+        <v>186</v>
+      </c>
+      <c r="E15" s="31" t="s">
+        <v>192</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>192</v>
-      </c>
-      <c r="G15" s="33">
+        <v>193</v>
+      </c>
+      <c r="G15" s="32">
         <v>3</v>
       </c>
       <c r="I15" s="14">
@@ -1802,7 +2170,7 @@
         <f t="shared" si="1"/>
         <v>6.6960000000000006</v>
       </c>
-      <c r="L15" s="25">
+      <c r="L15" s="24">
         <f t="shared" si="2"/>
         <v>5.58</v>
       </c>
@@ -1811,22 +2179,22 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.45">
       <c r="B16" t="s">
-        <v>263</v>
-      </c>
-      <c r="C16" s="32" t="s">
-        <v>197</v>
+        <v>264</v>
+      </c>
+      <c r="C16" s="31" t="s">
+        <v>198</v>
       </c>
       <c r="D16" t="s">
-        <v>185</v>
-      </c>
-      <c r="E16" s="32" t="s">
-        <v>200</v>
+        <v>186</v>
+      </c>
+      <c r="E16" s="31" t="s">
+        <v>201</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="G16" s="33">
-        <v>1</v>
+        <v>202</v>
+      </c>
+      <c r="G16" s="32">
+        <v>2</v>
       </c>
       <c r="I16" s="14">
         <f t="shared" si="0"/>
@@ -1837,33 +2205,33 @@
       </c>
       <c r="K16" s="14">
         <f t="shared" si="1"/>
-        <v>1.0920000000000001</v>
-      </c>
-      <c r="L16" s="25">
+        <v>2.1840000000000002</v>
+      </c>
+      <c r="L16" s="24">
         <f t="shared" si="2"/>
-        <v>0.91</v>
+        <v>1.82</v>
       </c>
       <c r="M16" s="16"/>
       <c r="N16" s="15"/>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B17" t="s">
-        <v>263</v>
-      </c>
-      <c r="C17" s="32" t="s">
-        <v>196</v>
+        <v>264</v>
+      </c>
+      <c r="C17" s="31" t="s">
+        <v>197</v>
       </c>
       <c r="D17" t="s">
-        <v>185</v>
-      </c>
-      <c r="E17" s="32" t="s">
-        <v>198</v>
+        <v>186</v>
+      </c>
+      <c r="E17" s="31" t="s">
+        <v>199</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>199</v>
-      </c>
-      <c r="G17" s="33">
-        <v>1</v>
+        <v>200</v>
+      </c>
+      <c r="G17" s="32">
+        <v>2</v>
       </c>
       <c r="I17" s="14">
         <f t="shared" si="0"/>
@@ -1874,32 +2242,32 @@
       </c>
       <c r="K17" s="14">
         <f t="shared" si="1"/>
-        <v>0.85199999999999998</v>
-      </c>
-      <c r="L17" s="25">
+        <v>1.704</v>
+      </c>
+      <c r="L17" s="24">
         <f t="shared" si="2"/>
-        <v>0.71</v>
+        <v>1.42</v>
       </c>
       <c r="M17" s="16"/>
       <c r="N17" s="15"/>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B18" t="s">
-        <v>263</v>
-      </c>
-      <c r="C18" s="32" t="s">
-        <v>182</v>
+        <v>264</v>
+      </c>
+      <c r="C18" s="31" t="s">
+        <v>183</v>
       </c>
       <c r="D18" t="s">
-        <v>185</v>
-      </c>
-      <c r="E18" s="32" t="s">
-        <v>202</v>
+        <v>186</v>
+      </c>
+      <c r="E18" s="31" t="s">
+        <v>203</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>203</v>
-      </c>
-      <c r="G18" s="33">
+        <v>204</v>
+      </c>
+      <c r="G18" s="32">
         <v>1</v>
       </c>
       <c r="I18" s="14">
@@ -1913,7 +2281,7 @@
         <f t="shared" si="1"/>
         <v>0.13200000000000001</v>
       </c>
-      <c r="L18" s="25">
+      <c r="L18" s="24">
         <f t="shared" si="2"/>
         <v>0.11</v>
       </c>
@@ -1922,21 +2290,21 @@
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B19" t="s">
-        <v>263</v>
-      </c>
-      <c r="C19" s="32" t="s">
-        <v>183</v>
+        <v>264</v>
+      </c>
+      <c r="C19" s="31" t="s">
+        <v>184</v>
       </c>
       <c r="D19" t="s">
-        <v>185</v>
-      </c>
-      <c r="E19" s="32" t="s">
-        <v>204</v>
+        <v>186</v>
+      </c>
+      <c r="E19" s="31" t="s">
+        <v>205</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>205</v>
-      </c>
-      <c r="G19" s="33">
+        <v>206</v>
+      </c>
+      <c r="G19" s="32">
         <v>1</v>
       </c>
       <c r="I19" s="14">
@@ -1950,7 +2318,7 @@
         <f t="shared" si="1"/>
         <v>0.13200000000000001</v>
       </c>
-      <c r="L19" s="25">
+      <c r="L19" s="24">
         <f t="shared" si="2"/>
         <v>0.11</v>
       </c>
@@ -1959,22 +2327,22 @@
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B20" t="s">
-        <v>263</v>
-      </c>
-      <c r="C20" s="32" t="s">
-        <v>206</v>
+        <v>264</v>
+      </c>
+      <c r="C20" s="31" t="s">
+        <v>207</v>
       </c>
       <c r="D20" t="s">
-        <v>185</v>
-      </c>
-      <c r="E20" s="32" t="s">
-        <v>207</v>
+        <v>186</v>
+      </c>
+      <c r="E20" s="31" t="s">
+        <v>208</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>208</v>
-      </c>
-      <c r="G20" s="33">
-        <v>1</v>
+        <v>209</v>
+      </c>
+      <c r="G20" s="32">
+        <v>2</v>
       </c>
       <c r="I20" s="14">
         <f t="shared" si="0"/>
@@ -1985,32 +2353,32 @@
       </c>
       <c r="K20" s="14">
         <f t="shared" si="1"/>
-        <v>3.0960000000000001</v>
-      </c>
-      <c r="L20" s="25">
+        <v>6.1920000000000002</v>
+      </c>
+      <c r="L20" s="24">
         <f t="shared" si="2"/>
-        <v>2.58</v>
+        <v>5.16</v>
       </c>
       <c r="M20" s="16"/>
       <c r="N20" s="15"/>
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B21" t="s">
-        <v>263</v>
-      </c>
-      <c r="C21" s="32" t="s">
-        <v>231</v>
+        <v>264</v>
+      </c>
+      <c r="C21" s="31" t="s">
+        <v>232</v>
       </c>
       <c r="D21" t="s">
-        <v>185</v>
-      </c>
-      <c r="E21" s="32" t="s">
+        <v>186</v>
+      </c>
+      <c r="E21" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="F21" s="13" t="s">
         <v>233</v>
       </c>
-      <c r="F21" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="G21" s="33">
+      <c r="G21" s="32">
         <v>2</v>
       </c>
       <c r="I21" s="14">
@@ -2024,7 +2392,7 @@
         <f t="shared" si="1"/>
         <v>0.98399999999999987</v>
       </c>
-      <c r="L21" s="25">
+      <c r="L21" s="24">
         <f t="shared" si="2"/>
         <v>0.82</v>
       </c>
@@ -2033,21 +2401,21 @@
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B22" t="s">
-        <v>263</v>
-      </c>
-      <c r="C22" s="32" t="s">
-        <v>234</v>
+        <v>264</v>
+      </c>
+      <c r="C22" s="31" t="s">
+        <v>235</v>
       </c>
       <c r="D22" t="s">
-        <v>185</v>
-      </c>
-      <c r="E22" s="32" t="s">
-        <v>236</v>
+        <v>186</v>
+      </c>
+      <c r="E22" s="31" t="s">
+        <v>237</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>237</v>
-      </c>
-      <c r="G22" s="33">
+        <v>238</v>
+      </c>
+      <c r="G22" s="32">
         <v>1</v>
       </c>
       <c r="I22" s="14">
@@ -2061,7 +2429,7 @@
         <f t="shared" si="1"/>
         <v>0.108</v>
       </c>
-      <c r="L22" s="25">
+      <c r="L22" s="24">
         <f t="shared" si="2"/>
         <v>0.09</v>
       </c>
@@ -2070,21 +2438,21 @@
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B23" t="s">
-        <v>263</v>
-      </c>
-      <c r="C23" s="32" t="s">
-        <v>243</v>
+        <v>264</v>
+      </c>
+      <c r="C23" s="31" t="s">
+        <v>244</v>
       </c>
       <c r="D23" t="s">
-        <v>185</v>
-      </c>
-      <c r="E23" s="32" t="s">
-        <v>244</v>
+        <v>186</v>
+      </c>
+      <c r="E23" s="31" t="s">
+        <v>245</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>245</v>
-      </c>
-      <c r="G23" s="33">
+        <v>246</v>
+      </c>
+      <c r="G23" s="32">
         <v>1</v>
       </c>
       <c r="I23" s="14">
@@ -2098,7 +2466,7 @@
         <f t="shared" si="1"/>
         <v>0.108</v>
       </c>
-      <c r="L23" s="25">
+      <c r="L23" s="24">
         <f t="shared" si="2"/>
         <v>0.09</v>
       </c>
@@ -2107,22 +2475,22 @@
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B24" t="s">
-        <v>263</v>
-      </c>
-      <c r="C24" s="32" t="s">
-        <v>246</v>
+        <v>264</v>
+      </c>
+      <c r="C24" s="31" t="s">
+        <v>247</v>
       </c>
       <c r="D24" t="s">
-        <v>185</v>
-      </c>
-      <c r="E24" s="32" t="s">
-        <v>247</v>
+        <v>186</v>
+      </c>
+      <c r="E24" s="31" t="s">
+        <v>248</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>248</v>
-      </c>
-      <c r="G24" s="33">
-        <v>2</v>
+        <v>249</v>
+      </c>
+      <c r="G24" s="32">
+        <v>8</v>
       </c>
       <c r="I24" s="14">
         <f t="shared" si="0"/>
@@ -2133,32 +2501,32 @@
       </c>
       <c r="K24" s="14">
         <f t="shared" si="1"/>
-        <v>0.216</v>
-      </c>
-      <c r="L24" s="25">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="L24" s="24">
         <f t="shared" si="2"/>
-        <v>0.18</v>
+        <v>0.72</v>
       </c>
       <c r="M24" s="16"/>
       <c r="N24" s="15"/>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B25" t="s">
-        <v>263</v>
-      </c>
-      <c r="C25" s="32" t="s">
-        <v>177</v>
+        <v>264</v>
+      </c>
+      <c r="C25" s="31" t="s">
+        <v>178</v>
       </c>
       <c r="D25" t="s">
-        <v>185</v>
-      </c>
-      <c r="E25" s="32" t="s">
-        <v>238</v>
+        <v>186</v>
+      </c>
+      <c r="E25" s="31" t="s">
+        <v>239</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>239</v>
-      </c>
-      <c r="G25" s="33">
+        <v>240</v>
+      </c>
+      <c r="G25" s="32">
         <v>1</v>
       </c>
       <c r="I25" s="14">
@@ -2172,7 +2540,7 @@
         <f t="shared" si="1"/>
         <v>0.108</v>
       </c>
-      <c r="L25" s="25">
+      <c r="L25" s="24">
         <f t="shared" si="2"/>
         <v>0.09</v>
       </c>
@@ -2181,21 +2549,21 @@
     </row>
     <row r="26" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B26" t="s">
-        <v>263</v>
-      </c>
-      <c r="C26" s="32" t="s">
-        <v>193</v>
+        <v>264</v>
+      </c>
+      <c r="C26" s="31" t="s">
+        <v>194</v>
       </c>
       <c r="D26" t="s">
-        <v>185</v>
-      </c>
-      <c r="E26" s="32" t="s">
-        <v>194</v>
+        <v>186</v>
+      </c>
+      <c r="E26" s="31" t="s">
+        <v>195</v>
       </c>
       <c r="F26" s="19" t="s">
-        <v>195</v>
-      </c>
-      <c r="G26" s="33">
+        <v>196</v>
+      </c>
+      <c r="G26" s="32">
         <v>1</v>
       </c>
       <c r="I26" s="14">
@@ -2209,7 +2577,7 @@
         <f t="shared" si="1"/>
         <v>6.48</v>
       </c>
-      <c r="L26" s="25">
+      <c r="L26" s="24">
         <f t="shared" si="2"/>
         <v>5.4</v>
       </c>
@@ -2218,19 +2586,19 @@
     </row>
     <row r="27" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B27" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C27" s="36" t="s">
+        <v>243</v>
+      </c>
+      <c r="D27" t="s">
+        <v>186</v>
+      </c>
+      <c r="E27" s="31" t="s">
+        <v>241</v>
+      </c>
+      <c r="F27" s="19" t="s">
         <v>242</v>
-      </c>
-      <c r="D27" t="s">
-        <v>185</v>
-      </c>
-      <c r="E27" s="32" t="s">
-        <v>240</v>
-      </c>
-      <c r="F27" s="19" t="s">
-        <v>241</v>
       </c>
       <c r="G27" s="37">
         <v>1</v>
@@ -2246,7 +2614,7 @@
         <f t="shared" si="1"/>
         <v>3.1799999999999997</v>
       </c>
-      <c r="L27" s="25">
+      <c r="L27" s="24">
         <f t="shared" si="2"/>
         <v>2.65</v>
       </c>
@@ -2255,35 +2623,35 @@
     </row>
     <row r="28" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B28" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C28" s="36" t="s">
+        <v>252</v>
+      </c>
+      <c r="D28" t="s">
+        <v>186</v>
+      </c>
+      <c r="E28" s="31" t="s">
+        <v>250</v>
+      </c>
+      <c r="F28" s="19" t="s">
         <v>251</v>
       </c>
-      <c r="D28" t="s">
-        <v>185</v>
-      </c>
-      <c r="E28" s="32" t="s">
-        <v>249</v>
-      </c>
-      <c r="F28" s="19" t="s">
-        <v>250</v>
-      </c>
-      <c r="G28" s="28">
+      <c r="G28" s="27">
         <v>48</v>
       </c>
       <c r="I28" s="14">
         <f t="shared" si="0"/>
         <v>0.192</v>
       </c>
-      <c r="J28" s="25">
+      <c r="J28" s="24">
         <v>0.16</v>
       </c>
       <c r="K28" s="14">
         <f t="shared" si="1"/>
         <v>9.2160000000000011</v>
       </c>
-      <c r="L28" s="25">
+      <c r="L28" s="24">
         <f t="shared" si="2"/>
         <v>7.68</v>
       </c>
@@ -2292,35 +2660,35 @@
     </row>
     <row r="29" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B29" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C29" s="36" t="s">
+        <v>255</v>
+      </c>
+      <c r="D29" t="s">
+        <v>186</v>
+      </c>
+      <c r="E29" s="31" t="s">
+        <v>253</v>
+      </c>
+      <c r="F29" s="19" t="s">
         <v>254</v>
       </c>
-      <c r="D29" t="s">
-        <v>185</v>
-      </c>
-      <c r="E29" s="32" t="s">
-        <v>252</v>
-      </c>
-      <c r="F29" s="19" t="s">
-        <v>253</v>
-      </c>
-      <c r="G29" s="28">
+      <c r="G29" s="27">
         <v>1</v>
       </c>
       <c r="I29" s="14">
         <f>J29*1.2</f>
         <v>2.1</v>
       </c>
-      <c r="J29" s="25">
+      <c r="J29" s="24">
         <v>1.75</v>
       </c>
       <c r="K29" s="14">
         <f>I29*G29</f>
         <v>2.1</v>
       </c>
-      <c r="L29" s="25">
+      <c r="L29" s="24">
         <f>J29*G29</f>
         <v>1.75</v>
       </c>
@@ -2330,75 +2698,75 @@
     </row>
     <row r="30" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C30" t="s">
+        <v>258</v>
+      </c>
+      <c r="D30" t="s">
         <v>257</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" s="31" t="s">
         <v>256</v>
       </c>
-      <c r="E30" s="32" t="s">
-        <v>255</v>
-      </c>
       <c r="F30" s="19" t="s">
-        <v>258</v>
-      </c>
-      <c r="G30" s="28">
+        <v>259</v>
+      </c>
+      <c r="G30" s="27">
         <v>2</v>
       </c>
       <c r="I30" s="14">
         <f>J30*1.2</f>
         <v>3.12</v>
       </c>
-      <c r="J30" s="25">
+      <c r="J30" s="24">
         <v>2.6</v>
       </c>
       <c r="K30" s="14">
         <f>I30*G30</f>
         <v>6.24</v>
       </c>
-      <c r="L30" s="25">
+      <c r="L30" s="24">
         <f>J30*G30</f>
         <v>5.2</v>
       </c>
       <c r="M30" s="16"/>
       <c r="N30" s="15"/>
       <c r="O30" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="31" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B31" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C31" t="s">
+        <v>262</v>
+      </c>
+      <c r="D31" t="s">
+        <v>186</v>
+      </c>
+      <c r="E31" s="31" t="s">
+        <v>263</v>
+      </c>
+      <c r="F31" s="39" t="s">
         <v>261</v>
       </c>
-      <c r="D31" t="s">
-        <v>185</v>
-      </c>
-      <c r="E31" s="32" t="s">
-        <v>262</v>
-      </c>
-      <c r="F31" s="39" t="s">
-        <v>260</v>
-      </c>
-      <c r="G31" s="28">
+      <c r="G31" s="27">
         <v>10</v>
       </c>
       <c r="I31" s="14">
         <f>J31*1.2</f>
         <v>1.92</v>
       </c>
-      <c r="J31" s="25">
+      <c r="J31" s="24">
         <v>1.6</v>
       </c>
       <c r="K31" s="14">
         <f>I31*G31</f>
         <v>19.2</v>
       </c>
-      <c r="L31" s="25">
+      <c r="L31" s="24">
         <f>J31*G31</f>
         <v>16</v>
       </c>
@@ -2406,202 +2774,1649 @@
       <c r="N31" s="15"/>
     </row>
     <row r="32" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B32" t="s">
+        <v>268</v>
+      </c>
+      <c r="C32" t="s">
+        <v>269</v>
+      </c>
+      <c r="D32" t="s">
+        <v>186</v>
+      </c>
+      <c r="E32" s="31" t="s">
+        <v>270</v>
+      </c>
+      <c r="F32" t="s">
+        <v>271</v>
+      </c>
+      <c r="G32" s="27">
+        <v>1</v>
+      </c>
+      <c r="I32" s="14">
+        <f>J32*1.2</f>
+        <v>3</v>
+      </c>
+      <c r="J32" s="24">
+        <v>2.5</v>
+      </c>
+      <c r="K32" s="14">
+        <f>I32*G32</f>
+        <v>3</v>
+      </c>
+      <c r="L32" s="24">
+        <f>J32*G32</f>
+        <v>2.5</v>
+      </c>
       <c r="M32" s="16"/>
       <c r="N32" s="15"/>
     </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="E33" s="32"/>
-      <c r="F33" s="19"/>
-      <c r="I33" s="14"/>
-      <c r="J33" s="25"/>
-      <c r="K33" s="14"/>
-      <c r="L33" s="25"/>
+    <row r="33" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B33" t="s">
+        <v>268</v>
+      </c>
+      <c r="C33" t="s">
+        <v>252</v>
+      </c>
+      <c r="D33" t="s">
+        <v>186</v>
+      </c>
+      <c r="E33" s="31" t="s">
+        <v>272</v>
+      </c>
+      <c r="F33" s="19" t="s">
+        <v>273</v>
+      </c>
+      <c r="G33" s="27">
+        <v>11</v>
+      </c>
+      <c r="I33" s="14">
+        <f>J33*1.2</f>
+        <v>0.68399999999999994</v>
+      </c>
+      <c r="J33" s="24">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="K33" s="14">
+        <f>I33*G33</f>
+        <v>7.5239999999999991</v>
+      </c>
+      <c r="L33" s="24">
+        <f>J33*G33</f>
+        <v>6.27</v>
+      </c>
       <c r="M33" s="16"/>
       <c r="N33" s="15"/>
     </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="E34" s="24"/>
-      <c r="F34" s="19"/>
-      <c r="I34" s="14"/>
-      <c r="J34" s="25"/>
-      <c r="K34" s="14"/>
-      <c r="L34" s="25"/>
+    <row r="34" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B34" t="s">
+        <v>268</v>
+      </c>
+      <c r="C34" t="s">
+        <v>276</v>
+      </c>
+      <c r="D34" t="s">
+        <v>186</v>
+      </c>
+      <c r="E34" s="31" t="s">
+        <v>274</v>
+      </c>
+      <c r="F34" s="19" t="s">
+        <v>275</v>
+      </c>
+      <c r="G34" s="27">
+        <v>2</v>
+      </c>
+      <c r="I34" s="14">
+        <f t="shared" ref="I34:I74" si="3">J34*1.2</f>
+        <v>0.68399999999999994</v>
+      </c>
+      <c r="J34" s="24">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="K34" s="14">
+        <f t="shared" ref="K34:K74" si="4">I34*G34</f>
+        <v>1.3679999999999999</v>
+      </c>
+      <c r="L34" s="24">
+        <f t="shared" ref="L34:L74" si="5">J34*G34</f>
+        <v>1.1399999999999999</v>
+      </c>
       <c r="M34" s="16"/>
       <c r="N34" s="15"/>
     </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="E35" s="24"/>
-      <c r="F35" s="13"/>
-      <c r="I35" s="14"/>
-      <c r="J35" s="25"/>
-      <c r="K35" s="14"/>
-      <c r="L35" s="25"/>
+    <row r="35" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B35" t="s">
+        <v>268</v>
+      </c>
+      <c r="C35" t="s">
+        <v>278</v>
+      </c>
+      <c r="D35" t="s">
+        <v>186</v>
+      </c>
+      <c r="E35" s="31" t="s">
+        <v>277</v>
+      </c>
+      <c r="F35" s="13" t="s">
+        <v>279</v>
+      </c>
+      <c r="G35" s="27">
+        <v>2</v>
+      </c>
+      <c r="I35" s="14">
+        <f t="shared" si="3"/>
+        <v>0.20400000000000001</v>
+      </c>
+      <c r="J35" s="24">
+        <v>0.17</v>
+      </c>
+      <c r="K35" s="14">
+        <f t="shared" si="4"/>
+        <v>0.40800000000000003</v>
+      </c>
+      <c r="L35" s="24">
+        <f t="shared" si="5"/>
+        <v>0.34</v>
+      </c>
       <c r="M35" s="16"/>
       <c r="N35" s="15"/>
     </row>
-    <row r="36" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="E36" s="24"/>
-      <c r="F36" s="19"/>
-      <c r="I36" s="14"/>
-      <c r="J36" s="25"/>
-      <c r="K36" s="14"/>
-      <c r="L36" s="25"/>
+    <row r="36" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B36" t="s">
+        <v>268</v>
+      </c>
+      <c r="C36" t="s">
+        <v>282</v>
+      </c>
+      <c r="D36" t="s">
+        <v>186</v>
+      </c>
+      <c r="E36" s="31" t="s">
+        <v>280</v>
+      </c>
+      <c r="F36" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="G36" s="27">
+        <v>4</v>
+      </c>
+      <c r="I36" s="14">
+        <f t="shared" si="3"/>
+        <v>0.16800000000000001</v>
+      </c>
+      <c r="J36" s="24">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="K36" s="14">
+        <f t="shared" si="4"/>
+        <v>0.67200000000000004</v>
+      </c>
+      <c r="L36" s="24">
+        <f t="shared" si="5"/>
+        <v>0.56000000000000005</v>
+      </c>
       <c r="M36" s="16"/>
       <c r="N36" s="15"/>
     </row>
-    <row r="37" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="E37" s="18"/>
-      <c r="F37" s="19"/>
-      <c r="I37" s="14"/>
-      <c r="J37" s="25"/>
-      <c r="K37" s="14"/>
-      <c r="L37" s="25"/>
+    <row r="37" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B37" t="s">
+        <v>268</v>
+      </c>
+      <c r="C37" t="s">
+        <v>285</v>
+      </c>
+      <c r="D37" t="s">
+        <v>186</v>
+      </c>
+      <c r="E37" s="31" t="s">
+        <v>283</v>
+      </c>
+      <c r="F37" s="19" t="s">
+        <v>284</v>
+      </c>
+      <c r="G37" s="27">
+        <v>1</v>
+      </c>
+      <c r="I37" s="14">
+        <f t="shared" si="3"/>
+        <v>0.33600000000000002</v>
+      </c>
+      <c r="J37" s="24">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="K37" s="14">
+        <f t="shared" si="4"/>
+        <v>0.33600000000000002</v>
+      </c>
+      <c r="L37" s="24">
+        <f t="shared" si="5"/>
+        <v>0.28000000000000003</v>
+      </c>
       <c r="M37" s="16"/>
       <c r="N37" s="15"/>
     </row>
-    <row r="38" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="E38" s="18"/>
-      <c r="F38" s="19"/>
-      <c r="I38" s="14"/>
-      <c r="J38" s="25"/>
-      <c r="K38" s="14"/>
-      <c r="L38" s="25"/>
+    <row r="38" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B38" t="s">
+        <v>268</v>
+      </c>
+      <c r="C38" t="s">
+        <v>286</v>
+      </c>
+      <c r="D38" t="s">
+        <v>186</v>
+      </c>
+      <c r="E38" s="31" t="s">
+        <v>287</v>
+      </c>
+      <c r="F38" s="19" t="s">
+        <v>288</v>
+      </c>
+      <c r="G38" s="27">
+        <v>3</v>
+      </c>
+      <c r="I38" s="14">
+        <f t="shared" si="3"/>
+        <v>0.88800000000000001</v>
+      </c>
+      <c r="J38" s="24">
+        <v>0.74</v>
+      </c>
+      <c r="K38" s="14">
+        <f t="shared" si="4"/>
+        <v>2.6640000000000001</v>
+      </c>
+      <c r="L38" s="24">
+        <f t="shared" si="5"/>
+        <v>2.2199999999999998</v>
+      </c>
       <c r="M38" s="16"/>
       <c r="N38" s="15"/>
     </row>
-    <row r="39" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="E39" s="18"/>
-      <c r="F39" s="19"/>
-      <c r="I39" s="14"/>
-      <c r="J39" s="25"/>
-      <c r="K39" s="14"/>
-      <c r="L39" s="25"/>
+    <row r="39" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B39" t="s">
+        <v>268</v>
+      </c>
+      <c r="C39" s="34" t="s">
+        <v>252</v>
+      </c>
+      <c r="D39" t="s">
+        <v>186</v>
+      </c>
+      <c r="E39" s="31" t="s">
+        <v>210</v>
+      </c>
+      <c r="F39" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="G39" s="27">
+        <v>2</v>
+      </c>
+      <c r="I39" s="14">
+        <f t="shared" si="3"/>
+        <v>0.156</v>
+      </c>
+      <c r="J39" s="24">
+        <v>0.13</v>
+      </c>
+      <c r="K39" s="14">
+        <f t="shared" si="4"/>
+        <v>0.312</v>
+      </c>
+      <c r="L39" s="24">
+        <f t="shared" si="5"/>
+        <v>0.26</v>
+      </c>
       <c r="M39" s="16"/>
       <c r="N39" s="15"/>
     </row>
-    <row r="40" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="E40" s="18"/>
-      <c r="F40" s="19"/>
-      <c r="I40" s="14"/>
-      <c r="J40" s="25"/>
-      <c r="K40" s="14"/>
-      <c r="L40" s="25"/>
+    <row r="40" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B40" t="s">
+        <v>268</v>
+      </c>
+      <c r="C40" t="s">
+        <v>285</v>
+      </c>
+      <c r="D40" t="s">
+        <v>186</v>
+      </c>
+      <c r="E40" s="31" t="s">
+        <v>290</v>
+      </c>
+      <c r="F40" s="19" t="s">
+        <v>291</v>
+      </c>
+      <c r="G40" s="27">
+        <v>3</v>
+      </c>
+      <c r="I40" s="14">
+        <f t="shared" si="3"/>
+        <v>0.16800000000000001</v>
+      </c>
+      <c r="J40" s="24">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="K40" s="14">
+        <f t="shared" si="4"/>
+        <v>0.504</v>
+      </c>
+      <c r="L40" s="24">
+        <f t="shared" si="5"/>
+        <v>0.42000000000000004</v>
+      </c>
       <c r="M40" s="16"/>
       <c r="N40" s="15"/>
     </row>
-    <row r="41" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="E41" s="18"/>
-      <c r="F41" s="19"/>
-      <c r="I41" s="14"/>
-      <c r="J41" s="25"/>
-      <c r="K41" s="14"/>
-      <c r="L41" s="25"/>
+    <row r="41" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B41" t="s">
+        <v>268</v>
+      </c>
+      <c r="C41" t="s">
+        <v>229</v>
+      </c>
+      <c r="D41" t="s">
+        <v>186</v>
+      </c>
+      <c r="E41" s="31" t="s">
+        <v>231</v>
+      </c>
+      <c r="F41" s="19" t="s">
+        <v>292</v>
+      </c>
+      <c r="G41" s="27">
+        <v>2</v>
+      </c>
+      <c r="I41" s="14">
+        <f t="shared" si="3"/>
+        <v>1.1279999999999999</v>
+      </c>
+      <c r="J41" s="24">
+        <v>0.94</v>
+      </c>
+      <c r="K41" s="14">
+        <f t="shared" si="4"/>
+        <v>2.2559999999999998</v>
+      </c>
+      <c r="L41" s="24">
+        <f t="shared" si="5"/>
+        <v>1.88</v>
+      </c>
       <c r="M41" s="16"/>
       <c r="N41" s="15"/>
     </row>
-    <row r="42" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="E42" s="18"/>
-      <c r="F42" s="19"/>
-      <c r="I42" s="14"/>
-      <c r="J42" s="25"/>
-      <c r="K42" s="14"/>
-      <c r="L42" s="25"/>
+    <row r="42" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B42" t="s">
+        <v>268</v>
+      </c>
+      <c r="C42" t="s">
+        <v>295</v>
+      </c>
+      <c r="D42" t="s">
+        <v>186</v>
+      </c>
+      <c r="E42" s="31" t="s">
+        <v>293</v>
+      </c>
+      <c r="F42" s="13" t="s">
+        <v>294</v>
+      </c>
+      <c r="G42" s="27">
+        <v>2</v>
+      </c>
+      <c r="I42" s="14">
+        <f t="shared" si="3"/>
+        <v>0.40800000000000003</v>
+      </c>
+      <c r="J42" s="24">
+        <v>0.34</v>
+      </c>
+      <c r="K42" s="14">
+        <f t="shared" si="4"/>
+        <v>0.81600000000000006</v>
+      </c>
+      <c r="L42" s="24">
+        <f t="shared" si="5"/>
+        <v>0.68</v>
+      </c>
       <c r="M42" s="16"/>
       <c r="N42" s="15"/>
     </row>
-    <row r="43" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="E43" s="18"/>
-      <c r="F43" s="13"/>
-      <c r="I43" s="14"/>
-      <c r="J43" s="14"/>
-      <c r="K43" s="14"/>
-      <c r="L43" s="25"/>
+    <row r="43" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B43" t="s">
+        <v>268</v>
+      </c>
+      <c r="C43" t="s">
+        <v>297</v>
+      </c>
+      <c r="D43" t="s">
+        <v>186</v>
+      </c>
+      <c r="E43" s="31" t="s">
+        <v>296</v>
+      </c>
+      <c r="F43" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="G43" s="27">
+        <v>1</v>
+      </c>
+      <c r="I43" s="14">
+        <f t="shared" si="3"/>
+        <v>3.7199999999999998</v>
+      </c>
+      <c r="J43" s="14">
+        <v>3.1</v>
+      </c>
+      <c r="K43" s="14">
+        <f t="shared" si="4"/>
+        <v>3.7199999999999998</v>
+      </c>
+      <c r="L43" s="24">
+        <f t="shared" si="5"/>
+        <v>3.1</v>
+      </c>
       <c r="M43" s="16"/>
       <c r="N43" s="15"/>
     </row>
-    <row r="44" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="E44" s="18"/>
-      <c r="F44" s="19"/>
-      <c r="I44" s="14"/>
-      <c r="J44" s="14"/>
-      <c r="K44" s="14"/>
-      <c r="L44" s="25"/>
+    <row r="44" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B44" t="s">
+        <v>268</v>
+      </c>
+      <c r="C44" t="s">
+        <v>301</v>
+      </c>
+      <c r="D44" t="s">
+        <v>186</v>
+      </c>
+      <c r="E44" s="31" t="s">
+        <v>299</v>
+      </c>
+      <c r="F44" s="19" t="s">
+        <v>300</v>
+      </c>
+      <c r="G44" s="27">
+        <v>1</v>
+      </c>
+      <c r="I44" s="14">
+        <f t="shared" si="3"/>
+        <v>1.728</v>
+      </c>
+      <c r="J44" s="14">
+        <v>1.44</v>
+      </c>
+      <c r="K44" s="14">
+        <f t="shared" si="4"/>
+        <v>1.728</v>
+      </c>
+      <c r="L44" s="24">
+        <f t="shared" si="5"/>
+        <v>1.44</v>
+      </c>
       <c r="M44" s="16"/>
       <c r="N44" s="15"/>
     </row>
-    <row r="45" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="E45" s="18"/>
-      <c r="F45" s="19"/>
-      <c r="I45" s="14"/>
-      <c r="J45" s="14"/>
-      <c r="K45" s="14"/>
-      <c r="L45" s="25"/>
+    <row r="45" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B45" t="s">
+        <v>268</v>
+      </c>
+      <c r="C45" t="s">
+        <v>304</v>
+      </c>
+      <c r="D45" t="s">
+        <v>186</v>
+      </c>
+      <c r="E45" s="31" t="s">
+        <v>302</v>
+      </c>
+      <c r="F45" s="19" t="s">
+        <v>303</v>
+      </c>
+      <c r="G45" s="27">
+        <v>2</v>
+      </c>
+      <c r="I45" s="14">
+        <f t="shared" si="3"/>
+        <v>0.42</v>
+      </c>
+      <c r="J45" s="14">
+        <v>0.35</v>
+      </c>
+      <c r="K45" s="14">
+        <f t="shared" si="4"/>
+        <v>0.84</v>
+      </c>
+      <c r="L45" s="24">
+        <f t="shared" si="5"/>
+        <v>0.7</v>
+      </c>
       <c r="M45" s="16"/>
       <c r="N45" s="15"/>
     </row>
-    <row r="46" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="E46" s="24"/>
-      <c r="F46" s="19"/>
-      <c r="I46" s="14"/>
-      <c r="J46" s="14"/>
-      <c r="K46" s="14"/>
-      <c r="L46" s="25"/>
+    <row r="46" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B46" t="s">
+        <v>268</v>
+      </c>
+      <c r="C46" t="s">
+        <v>306</v>
+      </c>
+      <c r="D46" t="s">
+        <v>186</v>
+      </c>
+      <c r="E46" s="31" t="s">
+        <v>305</v>
+      </c>
+      <c r="F46" s="19" t="s">
+        <v>307</v>
+      </c>
+      <c r="G46" s="27">
+        <v>1</v>
+      </c>
+      <c r="I46" s="14">
+        <f t="shared" si="3"/>
+        <v>6.3119999999999994</v>
+      </c>
+      <c r="J46" s="14">
+        <v>5.26</v>
+      </c>
+      <c r="K46" s="14">
+        <f t="shared" si="4"/>
+        <v>6.3119999999999994</v>
+      </c>
+      <c r="L46" s="24">
+        <f t="shared" si="5"/>
+        <v>5.26</v>
+      </c>
       <c r="M46" s="16"/>
       <c r="N46" s="15"/>
     </row>
-    <row r="47" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
-      <c r="F47" s="6"/>
-      <c r="G47" s="30"/>
-      <c r="H47" s="2"/>
-      <c r="I47" s="26"/>
-      <c r="J47" s="26"/>
-      <c r="K47" s="26"/>
-      <c r="L47" s="27"/>
-      <c r="M47" s="12"/>
-      <c r="N47" s="12"/>
-      <c r="O47" s="2"/>
-    </row>
-    <row r="48" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="I48" s="3"/>
-      <c r="J48" s="3"/>
-      <c r="K48" s="5">
-        <f>SUBTOTAL(9, K4:K47)</f>
-        <v>75.312000000000012</v>
-      </c>
-      <c r="L48" s="5">
-        <f>SUBTOTAL(9, L4:L47)</f>
-        <v>62.760000000000005</v>
-      </c>
-      <c r="M48" s="5"/>
-      <c r="N48" s="17">
-        <f>SUBTOTAL(9, N4:N47)</f>
+    <row r="47" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B47" t="s">
+        <v>268</v>
+      </c>
+      <c r="C47" t="s">
+        <v>309</v>
+      </c>
+      <c r="D47" t="s">
+        <v>186</v>
+      </c>
+      <c r="E47" s="31" t="s">
+        <v>308</v>
+      </c>
+      <c r="F47" s="19" t="s">
+        <v>310</v>
+      </c>
+      <c r="G47" s="27">
+        <v>1</v>
+      </c>
+      <c r="I47" s="14">
+        <f t="shared" si="3"/>
+        <v>0.70799999999999996</v>
+      </c>
+      <c r="J47" s="14">
+        <v>0.59</v>
+      </c>
+      <c r="K47" s="14">
+        <f t="shared" si="4"/>
+        <v>0.70799999999999996</v>
+      </c>
+      <c r="L47" s="24">
+        <f t="shared" si="5"/>
+        <v>0.59</v>
+      </c>
+      <c r="M47" s="16"/>
+      <c r="N47" s="15"/>
+    </row>
+    <row r="48" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B48" t="s">
+        <v>268</v>
+      </c>
+      <c r="C48" t="s">
+        <v>311</v>
+      </c>
+      <c r="D48" t="s">
+        <v>186</v>
+      </c>
+      <c r="E48" s="31" t="s">
+        <v>221</v>
+      </c>
+      <c r="F48" s="19" t="s">
+        <v>312</v>
+      </c>
+      <c r="G48" s="27">
+        <v>1</v>
+      </c>
+      <c r="I48" s="14">
+        <f t="shared" si="3"/>
+        <v>0.72</v>
+      </c>
+      <c r="J48" s="14">
+        <v>0.6</v>
+      </c>
+      <c r="K48" s="14">
+        <f t="shared" si="4"/>
+        <v>0.72</v>
+      </c>
+      <c r="L48" s="24">
+        <f t="shared" si="5"/>
+        <v>0.6</v>
+      </c>
+      <c r="M48" s="16"/>
+      <c r="N48" s="15"/>
+    </row>
+    <row r="49" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B49" t="s">
+        <v>268</v>
+      </c>
+      <c r="C49" t="s">
+        <v>177</v>
+      </c>
+      <c r="D49" t="s">
+        <v>186</v>
+      </c>
+      <c r="E49" s="31" t="s">
+        <v>253</v>
+      </c>
+      <c r="F49" s="19" t="s">
+        <v>313</v>
+      </c>
+      <c r="G49" s="27">
+        <v>2</v>
+      </c>
+      <c r="I49" s="14">
+        <f t="shared" si="3"/>
+        <v>2.1</v>
+      </c>
+      <c r="J49" s="14">
+        <v>1.75</v>
+      </c>
+      <c r="K49" s="14">
+        <f t="shared" si="4"/>
+        <v>4.2</v>
+      </c>
+      <c r="L49" s="24">
+        <f t="shared" si="5"/>
+        <v>3.5</v>
+      </c>
+      <c r="M49" s="16"/>
+      <c r="N49" s="15"/>
+    </row>
+    <row r="50" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B50" t="s">
+        <v>268</v>
+      </c>
+      <c r="C50" t="s">
+        <v>314</v>
+      </c>
+      <c r="D50" t="s">
+        <v>186</v>
+      </c>
+      <c r="E50" s="31" t="s">
+        <v>315</v>
+      </c>
+      <c r="F50" s="19" t="s">
+        <v>316</v>
+      </c>
+      <c r="G50" s="27">
+        <v>1</v>
+      </c>
+      <c r="I50" s="14">
+        <f t="shared" si="3"/>
+        <v>0.93599999999999994</v>
+      </c>
+      <c r="J50" s="14">
+        <v>0.78</v>
+      </c>
+      <c r="K50" s="14">
+        <f t="shared" si="4"/>
+        <v>0.93599999999999994</v>
+      </c>
+      <c r="L50" s="24">
+        <f t="shared" si="5"/>
+        <v>0.78</v>
+      </c>
+      <c r="M50" s="16"/>
+      <c r="N50" s="15"/>
+    </row>
+    <row r="51" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B51" t="s">
+        <v>268</v>
+      </c>
+      <c r="C51" t="s">
+        <v>319</v>
+      </c>
+      <c r="D51" t="s">
+        <v>186</v>
+      </c>
+      <c r="E51" s="31" t="s">
+        <v>317</v>
+      </c>
+      <c r="F51" s="19" t="s">
+        <v>318</v>
+      </c>
+      <c r="G51" s="27">
+        <v>1</v>
+      </c>
+      <c r="I51" s="14">
+        <f t="shared" si="3"/>
+        <v>2.8919999999999999</v>
+      </c>
+      <c r="J51" s="14">
+        <v>2.41</v>
+      </c>
+      <c r="K51" s="14">
+        <f t="shared" si="4"/>
+        <v>2.8919999999999999</v>
+      </c>
+      <c r="L51" s="24">
+        <f t="shared" si="5"/>
+        <v>2.41</v>
+      </c>
+      <c r="M51" s="16"/>
+      <c r="N51" s="15"/>
+    </row>
+    <row r="52" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B52" t="s">
+        <v>268</v>
+      </c>
+      <c r="C52" t="s">
+        <v>322</v>
+      </c>
+      <c r="D52" t="s">
+        <v>186</v>
+      </c>
+      <c r="E52" s="31" t="s">
+        <v>320</v>
+      </c>
+      <c r="F52" s="19" t="s">
+        <v>321</v>
+      </c>
+      <c r="G52" s="27">
+        <v>1</v>
+      </c>
+      <c r="I52" s="14">
+        <f t="shared" si="3"/>
+        <v>0.54</v>
+      </c>
+      <c r="J52" s="14">
+        <v>0.45</v>
+      </c>
+      <c r="K52" s="14">
+        <f t="shared" si="4"/>
+        <v>0.54</v>
+      </c>
+      <c r="L52" s="24">
+        <f t="shared" si="5"/>
+        <v>0.45</v>
+      </c>
+      <c r="M52" s="16"/>
+      <c r="N52" s="15"/>
+    </row>
+    <row r="53" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B53" t="s">
+        <v>268</v>
+      </c>
+      <c r="C53" t="s">
+        <v>325</v>
+      </c>
+      <c r="D53" t="s">
+        <v>186</v>
+      </c>
+      <c r="E53" s="31" t="s">
+        <v>323</v>
+      </c>
+      <c r="F53" s="19" t="s">
+        <v>324</v>
+      </c>
+      <c r="G53" s="27">
+        <v>2</v>
+      </c>
+      <c r="I53" s="14">
+        <f t="shared" si="3"/>
+        <v>0.3</v>
+      </c>
+      <c r="J53" s="14">
+        <v>0.25</v>
+      </c>
+      <c r="K53" s="14">
+        <f t="shared" si="4"/>
+        <v>0.6</v>
+      </c>
+      <c r="L53" s="24">
+        <f t="shared" si="5"/>
+        <v>0.5</v>
+      </c>
+      <c r="M53" s="16"/>
+      <c r="N53" s="15"/>
+    </row>
+    <row r="54" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B54" t="s">
+        <v>268</v>
+      </c>
+      <c r="C54" t="s">
+        <v>328</v>
+      </c>
+      <c r="D54" t="s">
+        <v>186</v>
+      </c>
+      <c r="E54" s="31" t="s">
+        <v>326</v>
+      </c>
+      <c r="F54" s="19" t="s">
+        <v>327</v>
+      </c>
+      <c r="G54" s="27">
+        <v>1</v>
+      </c>
+      <c r="I54" s="14">
+        <f t="shared" si="3"/>
+        <v>1.452</v>
+      </c>
+      <c r="J54" s="14">
+        <v>1.21</v>
+      </c>
+      <c r="K54" s="14">
+        <f t="shared" si="4"/>
+        <v>1.452</v>
+      </c>
+      <c r="L54" s="24">
+        <f t="shared" si="5"/>
+        <v>1.21</v>
+      </c>
+      <c r="M54" s="16"/>
+      <c r="N54" s="15"/>
+    </row>
+    <row r="55" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B55" t="s">
+        <v>268</v>
+      </c>
+      <c r="C55" t="s">
+        <v>244</v>
+      </c>
+      <c r="D55" t="s">
+        <v>186</v>
+      </c>
+      <c r="E55" s="31" t="s">
+        <v>329</v>
+      </c>
+      <c r="F55" s="19" t="s">
+        <v>330</v>
+      </c>
+      <c r="G55" s="27">
+        <v>2</v>
+      </c>
+      <c r="I55" s="14">
+        <f t="shared" si="3"/>
+        <v>1.1279999999999999</v>
+      </c>
+      <c r="J55" s="14">
+        <v>0.94</v>
+      </c>
+      <c r="K55" s="14">
+        <f t="shared" si="4"/>
+        <v>2.2559999999999998</v>
+      </c>
+      <c r="L55" s="24">
+        <f t="shared" si="5"/>
+        <v>1.88</v>
+      </c>
+      <c r="M55" s="16"/>
+      <c r="N55" s="15"/>
+    </row>
+    <row r="56" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B56" t="s">
+        <v>268</v>
+      </c>
+      <c r="C56" t="s">
+        <v>232</v>
+      </c>
+      <c r="D56" t="s">
+        <v>186</v>
+      </c>
+      <c r="E56" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="F56" s="19" t="s">
+        <v>331</v>
+      </c>
+      <c r="G56" s="27">
+        <v>3</v>
+      </c>
+      <c r="I56" s="14">
+        <f t="shared" si="3"/>
+        <v>0.49199999999999994</v>
+      </c>
+      <c r="J56" s="14">
+        <v>0.41</v>
+      </c>
+      <c r="K56" s="14">
+        <f t="shared" si="4"/>
+        <v>1.4759999999999998</v>
+      </c>
+      <c r="L56" s="24">
+        <f t="shared" si="5"/>
+        <v>1.23</v>
+      </c>
+      <c r="M56" s="16"/>
+      <c r="N56" s="15"/>
+    </row>
+    <row r="57" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B57" t="s">
+        <v>268</v>
+      </c>
+      <c r="C57" t="s">
+        <v>333</v>
+      </c>
+      <c r="D57" t="s">
+        <v>186</v>
+      </c>
+      <c r="E57" s="31" t="s">
+        <v>332</v>
+      </c>
+      <c r="F57" s="19" t="s">
+        <v>334</v>
+      </c>
+      <c r="G57" s="27">
+        <v>2</v>
+      </c>
+      <c r="I57" s="14">
+        <f t="shared" si="3"/>
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="J57" s="14">
+        <v>0.23</v>
+      </c>
+      <c r="K57" s="14">
+        <f t="shared" si="4"/>
+        <v>0.55200000000000005</v>
+      </c>
+      <c r="L57" s="24">
+        <f t="shared" si="5"/>
+        <v>0.46</v>
+      </c>
+      <c r="M57" s="16"/>
+      <c r="N57" s="15"/>
+    </row>
+    <row r="58" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B58" t="s">
+        <v>268</v>
+      </c>
+      <c r="C58" t="s">
+        <v>336</v>
+      </c>
+      <c r="D58" t="s">
+        <v>186</v>
+      </c>
+      <c r="E58" s="31" t="s">
+        <v>237</v>
+      </c>
+      <c r="F58" s="19" t="s">
+        <v>335</v>
+      </c>
+      <c r="G58" s="27">
+        <v>1</v>
+      </c>
+      <c r="I58" s="14">
+        <f t="shared" si="3"/>
+        <v>0.108</v>
+      </c>
+      <c r="J58" s="14">
+        <v>0.09</v>
+      </c>
+      <c r="K58" s="14">
+        <f t="shared" si="4"/>
+        <v>0.108</v>
+      </c>
+      <c r="L58" s="24">
+        <f t="shared" si="5"/>
+        <v>0.09</v>
+      </c>
+      <c r="M58" s="16"/>
+      <c r="N58" s="15"/>
+    </row>
+    <row r="59" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B59" t="s">
+        <v>268</v>
+      </c>
+      <c r="C59" t="s">
+        <v>339</v>
+      </c>
+      <c r="D59" t="s">
+        <v>186</v>
+      </c>
+      <c r="E59" s="31" t="s">
+        <v>337</v>
+      </c>
+      <c r="F59" s="19" t="s">
+        <v>338</v>
+      </c>
+      <c r="G59" s="27">
+        <v>2</v>
+      </c>
+      <c r="I59" s="14">
+        <f t="shared" si="3"/>
+        <v>0.13200000000000001</v>
+      </c>
+      <c r="J59" s="14">
+        <v>0.11</v>
+      </c>
+      <c r="K59" s="14">
+        <f t="shared" si="4"/>
+        <v>0.26400000000000001</v>
+      </c>
+      <c r="L59" s="24">
+        <f t="shared" si="5"/>
+        <v>0.22</v>
+      </c>
+      <c r="M59" s="16"/>
+      <c r="N59" s="15"/>
+    </row>
+    <row r="60" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B60" t="s">
+        <v>268</v>
+      </c>
+      <c r="C60" t="s">
+        <v>342</v>
+      </c>
+      <c r="D60" t="s">
+        <v>186</v>
+      </c>
+      <c r="E60" s="31" t="s">
+        <v>340</v>
+      </c>
+      <c r="F60" s="19" t="s">
+        <v>341</v>
+      </c>
+      <c r="G60" s="27">
+        <v>1</v>
+      </c>
+      <c r="I60" s="14">
+        <f t="shared" si="3"/>
+        <v>0.108</v>
+      </c>
+      <c r="J60" s="14">
+        <v>0.09</v>
+      </c>
+      <c r="K60" s="14">
+        <f t="shared" si="4"/>
+        <v>0.108</v>
+      </c>
+      <c r="L60" s="24">
+        <f t="shared" si="5"/>
+        <v>0.09</v>
+      </c>
+      <c r="M60" s="16"/>
+      <c r="N60" s="15"/>
+    </row>
+    <row r="61" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B61" t="s">
+        <v>268</v>
+      </c>
+      <c r="C61" t="s">
+        <v>345</v>
+      </c>
+      <c r="D61" t="s">
+        <v>186</v>
+      </c>
+      <c r="E61" s="31" t="s">
+        <v>343</v>
+      </c>
+      <c r="F61" s="19" t="s">
+        <v>344</v>
+      </c>
+      <c r="G61" s="27">
+        <v>1</v>
+      </c>
+      <c r="I61" s="14">
+        <f t="shared" si="3"/>
+        <v>0.12</v>
+      </c>
+      <c r="J61" s="14">
+        <v>0.1</v>
+      </c>
+      <c r="K61" s="14">
+        <f t="shared" si="4"/>
+        <v>0.12</v>
+      </c>
+      <c r="L61" s="24">
+        <f t="shared" si="5"/>
+        <v>0.1</v>
+      </c>
+      <c r="M61" s="16"/>
+      <c r="N61" s="15"/>
+    </row>
+    <row r="62" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B62" t="s">
+        <v>268</v>
+      </c>
+      <c r="C62" t="s">
+        <v>348</v>
+      </c>
+      <c r="D62" t="s">
+        <v>186</v>
+      </c>
+      <c r="E62" s="31" t="s">
+        <v>346</v>
+      </c>
+      <c r="F62" s="19" t="s">
+        <v>347</v>
+      </c>
+      <c r="G62" s="27">
+        <v>1</v>
+      </c>
+      <c r="I62" s="14">
+        <f t="shared" si="3"/>
+        <v>0.40800000000000003</v>
+      </c>
+      <c r="J62" s="14">
+        <v>0.34</v>
+      </c>
+      <c r="K62" s="14">
+        <f t="shared" si="4"/>
+        <v>0.40800000000000003</v>
+      </c>
+      <c r="L62" s="24">
+        <f t="shared" si="5"/>
+        <v>0.34</v>
+      </c>
+      <c r="M62" s="16"/>
+      <c r="N62" s="15"/>
+    </row>
+    <row r="63" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B63" t="s">
+        <v>268</v>
+      </c>
+      <c r="C63" t="s">
+        <v>351</v>
+      </c>
+      <c r="D63" t="s">
+        <v>186</v>
+      </c>
+      <c r="E63" s="31" t="s">
+        <v>349</v>
+      </c>
+      <c r="F63" s="19" t="s">
+        <v>350</v>
+      </c>
+      <c r="G63" s="27">
+        <v>1</v>
+      </c>
+      <c r="I63" s="14">
+        <f t="shared" si="3"/>
+        <v>0.108</v>
+      </c>
+      <c r="J63" s="14">
+        <v>0.09</v>
+      </c>
+      <c r="K63" s="14">
+        <f t="shared" si="4"/>
+        <v>0.108</v>
+      </c>
+      <c r="L63" s="24">
+        <f t="shared" si="5"/>
+        <v>0.09</v>
+      </c>
+      <c r="M63" s="16"/>
+      <c r="N63" s="15"/>
+    </row>
+    <row r="64" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B64" t="s">
+        <v>268</v>
+      </c>
+      <c r="C64" t="s">
+        <v>354</v>
+      </c>
+      <c r="D64" t="s">
+        <v>186</v>
+      </c>
+      <c r="E64" s="31" t="s">
+        <v>352</v>
+      </c>
+      <c r="F64" s="19" t="s">
+        <v>353</v>
+      </c>
+      <c r="G64" s="27">
+        <v>1</v>
+      </c>
+      <c r="I64" s="14">
+        <f t="shared" si="3"/>
+        <v>0.69599999999999995</v>
+      </c>
+      <c r="J64" s="14">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="K64" s="14">
+        <f t="shared" si="4"/>
+        <v>0.69599999999999995</v>
+      </c>
+      <c r="L64" s="24">
+        <f t="shared" si="5"/>
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="M64" s="16"/>
+      <c r="N64" s="15"/>
+    </row>
+    <row r="65" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B65" t="s">
+        <v>268</v>
+      </c>
+      <c r="C65" t="s">
+        <v>357</v>
+      </c>
+      <c r="D65" t="s">
+        <v>186</v>
+      </c>
+      <c r="E65" s="31" t="s">
+        <v>355</v>
+      </c>
+      <c r="F65" s="19" t="s">
+        <v>356</v>
+      </c>
+      <c r="G65" s="27">
+        <v>1</v>
+      </c>
+      <c r="I65" s="14">
+        <f t="shared" si="3"/>
+        <v>0.6</v>
+      </c>
+      <c r="J65" s="14">
+        <v>0.5</v>
+      </c>
+      <c r="K65" s="14">
+        <f t="shared" si="4"/>
+        <v>0.6</v>
+      </c>
+      <c r="L65" s="24">
+        <f t="shared" si="5"/>
+        <v>0.5</v>
+      </c>
+      <c r="M65" s="16"/>
+      <c r="N65" s="15"/>
+    </row>
+    <row r="66" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B66" t="s">
+        <v>268</v>
+      </c>
+      <c r="C66" t="s">
+        <v>359</v>
+      </c>
+      <c r="D66" t="s">
+        <v>186</v>
+      </c>
+      <c r="E66" s="31" t="s">
+        <v>239</v>
+      </c>
+      <c r="F66" s="19" t="s">
+        <v>358</v>
+      </c>
+      <c r="G66" s="27">
+        <v>1</v>
+      </c>
+      <c r="I66" s="14">
+        <f t="shared" si="3"/>
+        <v>0.108</v>
+      </c>
+      <c r="J66" s="14">
+        <v>0.09</v>
+      </c>
+      <c r="K66" s="14">
+        <f t="shared" si="4"/>
+        <v>0.108</v>
+      </c>
+      <c r="L66" s="24">
+        <f t="shared" si="5"/>
+        <v>0.09</v>
+      </c>
+      <c r="M66" s="16"/>
+      <c r="N66" s="15"/>
+    </row>
+    <row r="67" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B67" t="s">
+        <v>268</v>
+      </c>
+      <c r="C67" t="s">
+        <v>362</v>
+      </c>
+      <c r="D67" t="s">
+        <v>186</v>
+      </c>
+      <c r="E67" s="31" t="s">
+        <v>360</v>
+      </c>
+      <c r="F67" s="19" t="s">
+        <v>361</v>
+      </c>
+      <c r="G67" s="27">
+        <v>1</v>
+      </c>
+      <c r="I67" s="14">
+        <f t="shared" si="3"/>
+        <v>0.108</v>
+      </c>
+      <c r="J67" s="14">
+        <v>0.09</v>
+      </c>
+      <c r="K67" s="14">
+        <f t="shared" si="4"/>
+        <v>0.108</v>
+      </c>
+      <c r="L67" s="24">
+        <f t="shared" si="5"/>
+        <v>0.09</v>
+      </c>
+      <c r="M67" s="16"/>
+      <c r="N67" s="15"/>
+    </row>
+    <row r="68" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B68" t="s">
+        <v>268</v>
+      </c>
+      <c r="C68" t="s">
+        <v>365</v>
+      </c>
+      <c r="D68" t="s">
+        <v>186</v>
+      </c>
+      <c r="E68" s="31" t="s">
+        <v>363</v>
+      </c>
+      <c r="F68" t="s">
+        <v>364</v>
+      </c>
+      <c r="G68" s="27">
+        <v>2</v>
+      </c>
+      <c r="I68" s="14">
+        <f t="shared" si="3"/>
+        <v>0.108</v>
+      </c>
+      <c r="J68" s="14">
+        <v>0.09</v>
+      </c>
+      <c r="K68" s="14">
+        <f t="shared" si="4"/>
+        <v>0.216</v>
+      </c>
+      <c r="L68" s="24">
+        <f t="shared" si="5"/>
+        <v>0.18</v>
+      </c>
+      <c r="M68" s="16"/>
+      <c r="N68" s="15"/>
+    </row>
+    <row r="69" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B69" t="s">
+        <v>268</v>
+      </c>
+      <c r="C69" t="s">
+        <v>368</v>
+      </c>
+      <c r="D69" t="s">
+        <v>186</v>
+      </c>
+      <c r="E69" s="31" t="s">
+        <v>366</v>
+      </c>
+      <c r="F69" s="19" t="s">
+        <v>367</v>
+      </c>
+      <c r="G69" s="27">
+        <v>3</v>
+      </c>
+      <c r="I69" s="14">
+        <f t="shared" si="3"/>
+        <v>0.12</v>
+      </c>
+      <c r="J69" s="14">
+        <v>0.1</v>
+      </c>
+      <c r="K69" s="14">
+        <f t="shared" si="4"/>
+        <v>0.36</v>
+      </c>
+      <c r="L69" s="24">
+        <f t="shared" si="5"/>
+        <v>0.30000000000000004</v>
+      </c>
+      <c r="M69" s="16"/>
+      <c r="N69" s="15"/>
+    </row>
+    <row r="70" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B70" t="s">
+        <v>268</v>
+      </c>
+      <c r="C70" t="s">
+        <v>369</v>
+      </c>
+      <c r="D70" t="s">
+        <v>186</v>
+      </c>
+      <c r="E70" s="31" t="s">
+        <v>370</v>
+      </c>
+      <c r="F70" s="19" t="s">
+        <v>371</v>
+      </c>
+      <c r="G70" s="27">
+        <v>1</v>
+      </c>
+      <c r="I70" s="14">
+        <f t="shared" si="3"/>
+        <v>0.99599999999999989</v>
+      </c>
+      <c r="J70" s="14">
+        <v>0.83</v>
+      </c>
+      <c r="K70" s="14">
+        <f t="shared" si="4"/>
+        <v>0.99599999999999989</v>
+      </c>
+      <c r="L70" s="24">
+        <f t="shared" si="5"/>
+        <v>0.83</v>
+      </c>
+      <c r="M70" s="16"/>
+      <c r="N70" s="15"/>
+    </row>
+    <row r="71" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B71" t="s">
+        <v>268</v>
+      </c>
+      <c r="C71" t="s">
+        <v>374</v>
+      </c>
+      <c r="D71" t="s">
+        <v>186</v>
+      </c>
+      <c r="E71" s="31" t="s">
+        <v>372</v>
+      </c>
+      <c r="F71" s="19" t="s">
+        <v>373</v>
+      </c>
+      <c r="G71" s="27">
+        <v>1</v>
+      </c>
+      <c r="I71" s="14">
+        <f t="shared" si="3"/>
+        <v>7.032</v>
+      </c>
+      <c r="J71" s="14">
+        <v>5.86</v>
+      </c>
+      <c r="K71" s="14">
+        <f t="shared" si="4"/>
+        <v>7.032</v>
+      </c>
+      <c r="L71" s="24">
+        <f t="shared" si="5"/>
+        <v>5.86</v>
+      </c>
+      <c r="M71" s="16"/>
+      <c r="N71" s="15"/>
+    </row>
+    <row r="72" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B72" t="s">
+        <v>268</v>
+      </c>
+      <c r="C72" t="s">
+        <v>377</v>
+      </c>
+      <c r="D72" t="s">
+        <v>186</v>
+      </c>
+      <c r="E72" s="31" t="s">
+        <v>375</v>
+      </c>
+      <c r="F72" s="19" t="s">
+        <v>376</v>
+      </c>
+      <c r="G72" s="27">
+        <v>1</v>
+      </c>
+      <c r="I72" s="14">
+        <f t="shared" si="3"/>
+        <v>3.7199999999999998</v>
+      </c>
+      <c r="J72" s="14">
+        <v>3.1</v>
+      </c>
+      <c r="K72" s="14">
+        <f t="shared" si="4"/>
+        <v>3.7199999999999998</v>
+      </c>
+      <c r="L72" s="24">
+        <f t="shared" si="5"/>
+        <v>3.1</v>
+      </c>
+      <c r="M72" s="16"/>
+      <c r="N72" s="15"/>
+    </row>
+    <row r="73" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B73" t="s">
+        <v>268</v>
+      </c>
+      <c r="C73" t="s">
+        <v>177</v>
+      </c>
+      <c r="D73" t="s">
+        <v>378</v>
+      </c>
+      <c r="E73" s="31" t="s">
+        <v>379</v>
+      </c>
+      <c r="F73" s="19" t="s">
+        <v>380</v>
+      </c>
+      <c r="G73" s="27">
+        <v>4</v>
+      </c>
+      <c r="I73" s="14">
+        <f t="shared" si="3"/>
+        <v>2.2559999999999998</v>
+      </c>
+      <c r="J73" s="14">
+        <v>1.88</v>
+      </c>
+      <c r="K73" s="14">
+        <f t="shared" si="4"/>
+        <v>9.0239999999999991</v>
+      </c>
+      <c r="L73" s="24">
+        <f t="shared" si="5"/>
+        <v>7.52</v>
+      </c>
+      <c r="M73" s="16"/>
+      <c r="N73" s="15"/>
+    </row>
+    <row r="74" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B74" t="s">
+        <v>268</v>
+      </c>
+      <c r="C74" t="s">
+        <v>383</v>
+      </c>
+      <c r="D74" t="s">
+        <v>186</v>
+      </c>
+      <c r="E74" s="31" t="s">
+        <v>381</v>
+      </c>
+      <c r="F74" s="19" t="s">
+        <v>382</v>
+      </c>
+      <c r="G74" s="27">
+        <v>1</v>
+      </c>
+      <c r="I74" s="14">
+        <f t="shared" si="3"/>
+        <v>3.492</v>
+      </c>
+      <c r="J74" s="14">
+        <v>2.91</v>
+      </c>
+      <c r="K74" s="14">
+        <f t="shared" si="4"/>
+        <v>3.492</v>
+      </c>
+      <c r="L74" s="24">
+        <f t="shared" si="5"/>
+        <v>2.91</v>
+      </c>
+      <c r="M74" s="16"/>
+      <c r="N74" s="15"/>
+    </row>
+    <row r="75" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="B75" s="2"/>
+      <c r="C75" s="2"/>
+      <c r="E75" s="2"/>
+      <c r="F75" s="6"/>
+      <c r="G75" s="29"/>
+      <c r="H75" s="2"/>
+      <c r="I75" s="25"/>
+      <c r="J75" s="25"/>
+      <c r="K75" s="25"/>
+      <c r="L75" s="26"/>
+      <c r="M75" s="12"/>
+      <c r="N75" s="12"/>
+      <c r="O75" s="2"/>
+    </row>
+    <row r="76" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="D76" s="40"/>
+      <c r="I76" s="3"/>
+      <c r="J76" s="3"/>
+      <c r="K76" s="5">
+        <f>SUBTOTAL(9, K4:K75)</f>
+        <v>164.41200000000001</v>
+      </c>
+      <c r="L76" s="5">
+        <f>SUBTOTAL(9, L4:L75)</f>
+        <v>137.01000000000002</v>
+      </c>
+      <c r="M76" s="5"/>
+      <c r="N76" s="17">
+        <f>SUBTOTAL(9, N4:N75)</f>
         <v>0</v>
       </c>
-      <c r="O48" s="10" t="s">
+      <c r="O76" s="10" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="52" spans="4:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="D52" s="11"/>
-    </row>
-    <row r="55" spans="4:14" x14ac:dyDescent="0.45">
-      <c r="F55" s="7"/>
-      <c r="I55" s="8"/>
-      <c r="J55" s="8"/>
-      <c r="K55" s="8"/>
-      <c r="L55" s="8"/>
-      <c r="M55" s="8"/>
-      <c r="N55" s="8"/>
-    </row>
-    <row r="57" spans="4:14" x14ac:dyDescent="0.45">
-      <c r="F57" s="7"/>
-    </row>
-    <row r="64" spans="4:14" x14ac:dyDescent="0.45">
-      <c r="H64" s="9"/>
+    <row r="80" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="D80" s="11"/>
+    </row>
+    <row r="83" spans="6:14" x14ac:dyDescent="0.45">
+      <c r="F83" s="7"/>
+      <c r="I83" s="8"/>
+      <c r="J83" s="8"/>
+      <c r="K83" s="8"/>
+      <c r="L83" s="8"/>
+      <c r="M83" s="8"/>
+      <c r="N83" s="8"/>
+    </row>
+    <row r="85" spans="6:14" x14ac:dyDescent="0.45">
+      <c r="F85" s="7"/>
+    </row>
+    <row r="92" spans="6:14" x14ac:dyDescent="0.45">
+      <c r="H92" s="9"/>
     </row>
   </sheetData>
   <autoFilter ref="B3:O4" xr:uid="{00000000-0009-0000-0000-000000000000}"/>

</xml_diff>